<commit_message>
feat: update crawl 13/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R54fe58e31f08495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DAILY_CRAWL_PLAN" sheetId="2" r:id="R3cdb8accfe7749a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R97817e3b59e54739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="4" r:id="R9fbcac87a4a74ff9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUTOMATION_CONFIG" sheetId="5" r:id="R17b9984c950c4253"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R5c5f4a45d25e4dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R2cf56777cc574833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DAILY_CRAWL_PLAN" sheetId="2" r:id="Rc7e6632d28404e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R9ff1630eb4b442c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="4" r:id="R6a3d44cd1abf43df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUTOMATION_CONFIG" sheetId="5" r:id="Radbfcf24ea4e4576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R2cb7e2c44ca14371"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1229,7 +1229,7 @@
       </x:c>
       <x:c r="B10" s="175" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$C$4:$C$108,"Hoàn thành có lỗi")</x:f>
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1251,7 +1251,7 @@
       </x:c>
       <x:c r="B12" s="176" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!$C$4:$C$108,"Chưa chạy")</x:f>
-        <x:v>80</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="80" customFormat="1" ht="35" customHeight="1">
@@ -3417,7 +3417,7 @@
       </x:c>
       <x:c r="T29" s="125" t="str">
         <x:f>'CRAWL_LOG'!C29</x:f>
-        <x:v>Chưa chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="U29" s="86" t="inlineStr">
         <x:is>
@@ -3494,7 +3494,7 @@
       </x:c>
       <x:c r="T30" s="125" t="str">
         <x:f>'CRAWL_LOG'!C30</x:f>
-        <x:v>Chưa chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="U30" s="86" t="inlineStr">
         <x:is>
@@ -9521,7 +9521,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R770b92b95c4a4d01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a6030a9b7da4bce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11023,21 +11023,23 @@
           <x:t xml:space="preserve">00:30</x:t>
         </x:is>
       </x:c>
-      <x:c r="C26" t="str">
-        <x:v>Hoàn thành có lỗi</x:v>
+      <x:c r="C26" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn thành có lỗi</x:t>
+        </x:is>
       </x:c>
       <x:c r="D26" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="E26" s="180" t="n">
-        <x:v>46274.021689814814</x:v>
+        <x:v>46274.02168981481</x:v>
       </x:c>
       <x:c r="F26" s="180" t="n">
-        <x:v>46275.16547453703</x:v>
+        <x:v>46275.16547453704</x:v>
       </x:c>
       <x:c r="G26" s="181" t="n">
         <x:f>IF(OR(E26="",F26=""),"",(F26-E26)*24)</x:f>
-        <x:v>27.450833333248738</x:v>
+        <x:v>27.450833333597984</x:v>
       </x:c>
       <x:c r="H26" s="182" t="n">
         <x:v>4248</x:v>
@@ -11066,8 +11068,10 @@
       <x:c r="P26" s="182" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="Q26" s="86" t="str">
-        <x:v>Scheduled run 36 đã đạt terminal state; save_artifacts=false; scraper_version=2.3.0</x:v>
+      <x:c r="Q26" s="86" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Scheduled run 36 đã đạt terminal state; save_artifacts=false; scraper_version=2.3.0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="27" s="80" customFormat="1" ht="24" customHeight="1">
@@ -11155,11 +11159,11 @@
         <x:v>46276.0233637037</x:v>
       </x:c>
       <x:c r="F28" s="180" t="n">
-        <x:v>46276.85465078014</x:v>
+        <x:v>46276.85465077547</x:v>
       </x:c>
       <x:c r="G28" s="181" t="n">
         <x:f>IF(OR(E28="",F28=""),"",(F28-E28)*24)</x:f>
-        <x:v>19.950889834435657</x:v>
+        <x:v>19.950889722502325</x:v>
       </x:c>
       <x:c r="H28" s="182" t="n">
         <x:v>4248</x:v>
@@ -11205,26 +11209,56 @@
       </x:c>
       <x:c r="C29" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Chưa chạy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E29" s="180" t="n"/>
-      <x:c r="F29" s="180" t="n"/>
-      <x:c r="G29" s="181" t="str">
+          <x:t xml:space="preserve">Hoàn thành có lỗi</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">39</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E29" s="180" t="n">
+        <x:v>46277.0223231713</x:v>
+      </x:c>
+      <x:c r="F29" s="180" t="n">
+        <x:v>46277.68001267361</x:v>
+      </x:c>
+      <x:c r="G29" s="181" t="n">
         <x:f>IF(OR(E29="",F29=""),"",(F29-E29)*24)</x:f>
-      </x:c>
-      <x:c r="H29" s="182" t="n"/>
-      <x:c r="I29" s="182" t="n"/>
-      <x:c r="J29" s="182" t="n"/>
-      <x:c r="K29" s="182" t="n"/>
-      <x:c r="L29" s="182" t="n"/>
-      <x:c r="M29" s="182" t="n"/>
-      <x:c r="N29" s="182" t="n"/>
-      <x:c r="O29" s="182" t="n"/>
+        <x:v>15.78454805543879</x:v>
+      </x:c>
+      <x:c r="H29" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="I29" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="J29" s="182" t="n">
+        <x:v>3810</x:v>
+      </x:c>
+      <x:c r="K29" s="182" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="182" t="n">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="M29" s="182" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="N29" s="182" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="O29" s="182" t="n">
+        <x:v>34269</x:v>
+      </x:c>
       <x:c r="P29" s="182" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="Q29" s="86" t="n"/>
+      <x:c r="Q29" s="86" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Scheduled run 39 đã đạt terminal state</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="30" s="80" customFormat="1" ht="24" customHeight="1">
       <x:c r="A30" s="177" t="n">
@@ -11235,28 +11269,52 @@
           <x:t xml:space="preserve">00:30</x:t>
         </x:is>
       </x:c>
-      <x:c r="C30" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chưa chạy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="180" t="n"/>
-      <x:c r="F30" s="180" t="n"/>
-      <x:c r="G30" s="181" t="str">
+      <x:c r="C30" t="str">
+        <x:v>Hoàn thành có lỗi</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E30" s="180" t="n">
+        <x:v>46278.028969907406</x:v>
+      </x:c>
+      <x:c r="F30" s="180" t="n">
+        <x:v>46278.681122685186</x:v>
+      </x:c>
+      <x:c r="G30" s="181" t="n">
         <x:f>IF(OR(E30="",F30=""),"",(F30-E30)*24)</x:f>
-      </x:c>
-      <x:c r="H30" s="182" t="n"/>
-      <x:c r="I30" s="182" t="n"/>
-      <x:c r="J30" s="182" t="n"/>
-      <x:c r="K30" s="182" t="n"/>
-      <x:c r="L30" s="182" t="n"/>
-      <x:c r="M30" s="182" t="n"/>
-      <x:c r="N30" s="182" t="n"/>
-      <x:c r="O30" s="182" t="n"/>
+        <x:v>15.651666666730307</x:v>
+      </x:c>
+      <x:c r="H30" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="I30" s="182" t="n">
+        <x:v>4248</x:v>
+      </x:c>
+      <x:c r="J30" s="182" t="n">
+        <x:v>3844</x:v>
+      </x:c>
+      <x:c r="K30" s="182" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="182" t="n">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="M30" s="182" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="N30" s="182" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="O30" s="182" t="n">
+        <x:v>34617</x:v>
+      </x:c>
       <x:c r="P30" s="182" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="Q30" s="86" t="n"/>
+      <x:c r="Q30" s="86" t="str">
+        <x:v>Scheduled run 40 đã đạt terminal state; save_artifacts=false; scraper_version=2.3.0</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" s="80" customFormat="1" ht="24" customHeight="1">
       <x:c r="A31" s="177" t="n">
@@ -13774,7 +13832,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37386d5a855149d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9afa1ad8350a4e1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat: update crawl 16/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11358,7 +11358,7 @@
         <v>46279.01871327547</v>
       </c>
       <c r="F31" s="180" t="n">
-        <v>46279.67221261655</v>
+        <v>46279.67221261574</v>
       </c>
       <c r="G31" s="181">
         <f>IF(OR(E31="",F31=""),"",(F31-E31)*24)</f>
@@ -11408,27 +11408,56 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E32" s="180" t="n"/>
-      <c r="F32" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E32" s="180" t="n">
+        <v>46280.02255042824</v>
+      </c>
+      <c r="F32" s="180" t="n">
+        <v>46280.67743945602</v>
+      </c>
       <c r="G32" s="181">
         <f>IF(OR(E32="",F32=""),"",(F32-E32)*24)</f>
         <v/>
       </c>
-      <c r="H32" s="182" t="n"/>
-      <c r="I32" s="182" t="n"/>
-      <c r="J32" s="182" t="n"/>
-      <c r="K32" s="182" t="n"/>
-      <c r="L32" s="182" t="n"/>
-      <c r="M32" s="182" t="n"/>
-      <c r="N32" s="182" t="n"/>
-      <c r="O32" s="182" t="n"/>
+      <c r="H32" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I32" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J32" s="182" t="n">
+        <v>3819</v>
+      </c>
+      <c r="K32" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="182" t="n">
+        <v>357</v>
+      </c>
+      <c r="M32" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N32" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O32" s="182" t="n">
+        <v>34515</v>
+      </c>
       <c r="P32" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q32" s="86" t="n"/>
+      <c r="Q32" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 42 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="24" customHeight="1" s="80">
       <c r="A33" s="177" t="n">
@@ -11441,10 +11470,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E33" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E33" s="180" t="n">
+        <v>46281.02375913026</v>
+      </c>
       <c r="F33" s="180" t="n"/>
       <c r="G33" s="181">
         <f>IF(OR(E33="",F33=""),"",(F33-E33)*24)</f>
@@ -11461,7 +11497,11 @@
       <c r="P33" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q33" s="86" t="n"/>
+      <c r="Q33" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="24" customHeight="1" s="80">
       <c r="A34" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 17/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11482,7 +11482,7 @@
         <v>46281.02375913195</v>
       </c>
       <c r="F33" s="180" t="n">
-        <v>46281.68837626058</v>
+        <v>46281.68837626158</v>
       </c>
       <c r="G33" s="181">
         <f>IF(OR(E33="",F33=""),"",(F33-E33)*24)</f>
@@ -11532,27 +11532,56 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E34" s="180" t="n"/>
-      <c r="F34" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E34" s="180" t="n">
+        <v>46282.02366894676</v>
+      </c>
+      <c r="F34" s="180" t="n">
+        <v>46282.65633473373</v>
+      </c>
       <c r="G34" s="181">
         <f>IF(OR(E34="",F34=""),"",(F34-E34)*24)</f>
         <v/>
       </c>
-      <c r="H34" s="182" t="n"/>
-      <c r="I34" s="182" t="n"/>
-      <c r="J34" s="182" t="n"/>
-      <c r="K34" s="182" t="n"/>
-      <c r="L34" s="182" t="n"/>
-      <c r="M34" s="182" t="n"/>
-      <c r="N34" s="182" t="n"/>
-      <c r="O34" s="182" t="n"/>
+      <c r="H34" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I34" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J34" s="182" t="n">
+        <v>3755</v>
+      </c>
+      <c r="K34" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="182" t="n">
+        <v>361</v>
+      </c>
+      <c r="M34" s="182" t="n">
+        <v>108</v>
+      </c>
+      <c r="N34" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O34" s="182" t="n">
+        <v>32953</v>
+      </c>
       <c r="P34" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q34" s="86" t="n"/>
+      <c r="Q34" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 44 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="24" customHeight="1" s="80">
       <c r="A35" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 18/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11544,7 +11544,7 @@
         <v>46282.02366894676</v>
       </c>
       <c r="F34" s="180" t="n">
-        <v>46282.65633473373</v>
+        <v>46282.65633473379</v>
       </c>
       <c r="G34" s="181">
         <f>IF(OR(E34="",F34=""),"",(F34-E34)*24)</f>
@@ -11594,27 +11594,56 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E35" s="180" t="n"/>
-      <c r="F35" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E35" s="180" t="n">
+        <v>46283.02431011574</v>
+      </c>
+      <c r="F35" s="180" t="n">
+        <v>46283.66392142885</v>
+      </c>
       <c r="G35" s="181">
         <f>IF(OR(E35="",F35=""),"",(F35-E35)*24)</f>
         <v/>
       </c>
-      <c r="H35" s="182" t="n"/>
-      <c r="I35" s="182" t="n"/>
-      <c r="J35" s="182" t="n"/>
-      <c r="K35" s="182" t="n"/>
-      <c r="L35" s="182" t="n"/>
-      <c r="M35" s="182" t="n"/>
-      <c r="N35" s="182" t="n"/>
-      <c r="O35" s="182" t="n"/>
+      <c r="H35" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I35" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J35" s="182" t="n">
+        <v>3764</v>
+      </c>
+      <c r="K35" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="182" t="n">
+        <v>364</v>
+      </c>
+      <c r="M35" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N35" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O35" s="182" t="n">
+        <v>34805</v>
+      </c>
       <c r="P35" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q35" s="86" t="n"/>
+      <c r="Q35" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 45 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="24" customHeight="1" s="80">
       <c r="A36" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 19/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11606,7 +11606,7 @@
         <v>46283.02431011574</v>
       </c>
       <c r="F35" s="180" t="n">
-        <v>46283.66392142885</v>
+        <v>46283.66392142361</v>
       </c>
       <c r="G35" s="181">
         <f>IF(OR(E35="",F35=""),"",(F35-E35)*24)</f>
@@ -11656,27 +11656,56 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E36" s="180" t="n"/>
-      <c r="F36" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E36" s="180" t="n">
+        <v>46284.02278900463</v>
+      </c>
+      <c r="F36" s="180" t="n">
+        <v>46284.66309460479</v>
+      </c>
       <c r="G36" s="181">
         <f>IF(OR(E36="",F36=""),"",(F36-E36)*24)</f>
         <v/>
       </c>
-      <c r="H36" s="182" t="n"/>
-      <c r="I36" s="182" t="n"/>
-      <c r="J36" s="182" t="n"/>
-      <c r="K36" s="182" t="n"/>
-      <c r="L36" s="182" t="n"/>
-      <c r="M36" s="182" t="n"/>
-      <c r="N36" s="182" t="n"/>
-      <c r="O36" s="182" t="n"/>
+      <c r="H36" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I36" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J36" s="182" t="n">
+        <v>3767</v>
+      </c>
+      <c r="K36" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="182" t="n">
+        <v>397</v>
+      </c>
+      <c r="M36" s="182" t="n">
+        <v>60</v>
+      </c>
+      <c r="N36" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O36" s="182" t="n">
+        <v>34329</v>
+      </c>
       <c r="P36" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q36" s="86" t="n"/>
+      <c r="Q36" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 46 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="24" customHeight="1" s="80">
       <c r="A37" s="177" t="n">

</xml_diff>

<commit_message>
feat: start crawl 20/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11668,7 +11668,7 @@
         <v>46284.02278900463</v>
       </c>
       <c r="F36" s="180" t="n">
-        <v>46284.66309460479</v>
+        <v>46284.66309460648</v>
       </c>
       <c r="G36" s="181">
         <f>IF(OR(E36="",F36=""),"",(F36-E36)*24)</f>
@@ -11718,10 +11718,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E37" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="E37" s="180" t="n">
+        <v>46285.09141877551</v>
+      </c>
       <c r="F37" s="180" t="n"/>
       <c r="G37" s="181">
         <f>IF(OR(E37="",F37=""),"",(F37-E37)*24)</f>
@@ -11738,7 +11745,11 @@
       <c r="P37" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q37" s="86" t="n"/>
+      <c r="Q37" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="24" customHeight="1" s="80">
       <c r="A38" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 20/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11718,7 +11718,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -11727,27 +11727,45 @@
         </is>
       </c>
       <c r="E37" s="180" t="n">
-        <v>46285.09141877551</v>
-      </c>
-      <c r="F37" s="180" t="n"/>
+        <v>46285.09141877315</v>
+      </c>
+      <c r="F37" s="180" t="n">
+        <v>46285.7435316373</v>
+      </c>
       <c r="G37" s="181">
         <f>IF(OR(E37="",F37=""),"",(F37-E37)*24)</f>
         <v/>
       </c>
-      <c r="H37" s="182" t="n"/>
-      <c r="I37" s="182" t="n"/>
-      <c r="J37" s="182" t="n"/>
-      <c r="K37" s="182" t="n"/>
-      <c r="L37" s="182" t="n"/>
-      <c r="M37" s="182" t="n"/>
-      <c r="N37" s="182" t="n"/>
-      <c r="O37" s="182" t="n"/>
+      <c r="H37" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I37" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J37" s="182" t="n">
+        <v>3817</v>
+      </c>
+      <c r="K37" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="182" t="n">
+        <v>359</v>
+      </c>
+      <c r="M37" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N37" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O37" s="182" t="n">
+        <v>34172</v>
+      </c>
       <c r="P37" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q37" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 47 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 21/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11730,7 +11730,7 @@
         <v>46285.09141877315</v>
       </c>
       <c r="F37" s="180" t="n">
-        <v>46285.7435316373</v>
+        <v>46285.74353163195</v>
       </c>
       <c r="G37" s="181">
         <f>IF(OR(E37="",F37=""),"",(F37-E37)*24)</f>
@@ -11780,27 +11780,56 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E38" s="180" t="n"/>
-      <c r="F38" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E38" s="180" t="n">
+        <v>46286.02317181713</v>
+      </c>
+      <c r="F38" s="180" t="n">
+        <v>46286.66417160964</v>
+      </c>
       <c r="G38" s="181">
         <f>IF(OR(E38="",F38=""),"",(F38-E38)*24)</f>
         <v/>
       </c>
-      <c r="H38" s="182" t="n"/>
-      <c r="I38" s="182" t="n"/>
-      <c r="J38" s="182" t="n"/>
-      <c r="K38" s="182" t="n"/>
-      <c r="L38" s="182" t="n"/>
-      <c r="M38" s="182" t="n"/>
-      <c r="N38" s="182" t="n"/>
-      <c r="O38" s="182" t="n"/>
+      <c r="H38" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I38" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J38" s="182" t="n">
+        <v>3813</v>
+      </c>
+      <c r="K38" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="182" t="n">
+        <v>363</v>
+      </c>
+      <c r="M38" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N38" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O38" s="182" t="n">
+        <v>33015</v>
+      </c>
       <c r="P38" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q38" s="86" t="n"/>
+      <c r="Q38" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 48 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="24" customHeight="1" s="80">
       <c r="A39" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 22/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11792,7 +11792,7 @@
         <v>46286.02317181713</v>
       </c>
       <c r="F38" s="180" t="n">
-        <v>46286.66417160964</v>
+        <v>46286.6641716088</v>
       </c>
       <c r="G38" s="181">
         <f>IF(OR(E38="",F38=""),"",(F38-E38)*24)</f>
@@ -11842,27 +11842,56 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E39" s="180" t="n"/>
-      <c r="F39" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E39" s="180" t="n">
+        <v>46287.02362409722</v>
+      </c>
+      <c r="F39" s="180" t="n">
+        <v>46287.80768478286</v>
+      </c>
       <c r="G39" s="181">
         <f>IF(OR(E39="",F39=""),"",(F39-E39)*24)</f>
         <v/>
       </c>
-      <c r="H39" s="182" t="n"/>
-      <c r="I39" s="182" t="n"/>
-      <c r="J39" s="182" t="n"/>
-      <c r="K39" s="182" t="n"/>
-      <c r="L39" s="182" t="n"/>
-      <c r="M39" s="182" t="n"/>
-      <c r="N39" s="182" t="n"/>
-      <c r="O39" s="182" t="n"/>
+      <c r="H39" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I39" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J39" s="182" t="n">
+        <v>3776</v>
+      </c>
+      <c r="K39" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="182" t="n">
+        <v>400</v>
+      </c>
+      <c r="M39" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N39" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O39" s="182" t="n">
+        <v>34932</v>
+      </c>
       <c r="P39" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q39" s="86" t="n"/>
+      <c r="Q39" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 49 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="24" customHeight="1" s="80">
       <c r="A40" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 23/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11854,7 +11854,7 @@
         <v>46287.02362409722</v>
       </c>
       <c r="F39" s="180" t="n">
-        <v>46287.80768478286</v>
+        <v>46287.80768478009</v>
       </c>
       <c r="G39" s="181">
         <f>IF(OR(E39="",F39=""),"",(F39-E39)*24)</f>
@@ -11904,27 +11904,56 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E40" s="180" t="n"/>
-      <c r="F40" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E40" s="180" t="n">
+        <v>46288.02296778935</v>
+      </c>
+      <c r="F40" s="180" t="n">
+        <v>46288.66952380459</v>
+      </c>
       <c r="G40" s="181">
         <f>IF(OR(E40="",F40=""),"",(F40-E40)*24)</f>
         <v/>
       </c>
-      <c r="H40" s="182" t="n"/>
-      <c r="I40" s="182" t="n"/>
-      <c r="J40" s="182" t="n"/>
-      <c r="K40" s="182" t="n"/>
-      <c r="L40" s="182" t="n"/>
-      <c r="M40" s="182" t="n"/>
-      <c r="N40" s="182" t="n"/>
-      <c r="O40" s="182" t="n"/>
+      <c r="H40" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I40" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J40" s="182" t="n">
+        <v>3802</v>
+      </c>
+      <c r="K40" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="182" t="n">
+        <v>386</v>
+      </c>
+      <c r="M40" s="182" t="n">
+        <v>36</v>
+      </c>
+      <c r="N40" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O40" s="182" t="n">
+        <v>34399</v>
+      </c>
       <c r="P40" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q40" s="86" t="n"/>
+      <c r="Q40" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 50 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="24" customHeight="1" s="80">
       <c r="A41" s="177" t="n">

</xml_diff>

<commit_message>
feat: fix coverage matrix test
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11916,7 +11916,7 @@
         <v>46288.02296778935</v>
       </c>
       <c r="F40" s="180" t="n">
-        <v>46288.66952380459</v>
+        <v>46288.66952380787</v>
       </c>
       <c r="G40" s="181">
         <f>IF(OR(E40="",F40=""),"",(F40-E40)*24)</f>
@@ -11966,10 +11966,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E41" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="E41" s="180" t="n">
+        <v>46289.0232610831</v>
+      </c>
       <c r="F41" s="180" t="n"/>
       <c r="G41" s="181">
         <f>IF(OR(E41="",F41=""),"",(F41-E41)*24)</f>
@@ -11986,7 +11993,11 @@
       <c r="P41" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q41" s="86" t="n"/>
+      <c r="Q41" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="24" customHeight="1" s="80">
       <c r="A42" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 24/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11966,7 +11966,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -11975,27 +11975,45 @@
         </is>
       </c>
       <c r="E41" s="180" t="n">
-        <v>46289.0232610831</v>
-      </c>
-      <c r="F41" s="180" t="n"/>
+        <v>46289.02326108796</v>
+      </c>
+      <c r="F41" s="180" t="n">
+        <v>46289.65940128021</v>
+      </c>
       <c r="G41" s="181">
         <f>IF(OR(E41="",F41=""),"",(F41-E41)*24)</f>
         <v/>
       </c>
-      <c r="H41" s="182" t="n"/>
-      <c r="I41" s="182" t="n"/>
-      <c r="J41" s="182" t="n"/>
-      <c r="K41" s="182" t="n"/>
-      <c r="L41" s="182" t="n"/>
-      <c r="M41" s="182" t="n"/>
-      <c r="N41" s="182" t="n"/>
-      <c r="O41" s="182" t="n"/>
+      <c r="H41" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I41" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J41" s="182" t="n">
+        <v>3705</v>
+      </c>
+      <c r="K41" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="182" t="n">
+        <v>471</v>
+      </c>
+      <c r="M41" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N41" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O41" s="182" t="n">
+        <v>33753</v>
+      </c>
       <c r="P41" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q41" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 51 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 25/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -11978,7 +11978,7 @@
         <v>46289.02326108796</v>
       </c>
       <c r="F41" s="180" t="n">
-        <v>46289.65940128021</v>
+        <v>46289.65940128472</v>
       </c>
       <c r="G41" s="181">
         <f>IF(OR(E41="",F41=""),"",(F41-E41)*24)</f>
@@ -12028,27 +12028,56 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E42" s="180" t="n"/>
-      <c r="F42" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E42" s="180" t="n">
+        <v>46290.02230041667</v>
+      </c>
+      <c r="F42" s="180" t="n">
+        <v>46290.66399692127</v>
+      </c>
       <c r="G42" s="181">
         <f>IF(OR(E42="",F42=""),"",(F42-E42)*24)</f>
         <v/>
       </c>
-      <c r="H42" s="182" t="n"/>
-      <c r="I42" s="182" t="n"/>
-      <c r="J42" s="182" t="n"/>
-      <c r="K42" s="182" t="n"/>
-      <c r="L42" s="182" t="n"/>
-      <c r="M42" s="182" t="n"/>
-      <c r="N42" s="182" t="n"/>
-      <c r="O42" s="182" t="n"/>
+      <c r="H42" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I42" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J42" s="182" t="n">
+        <v>3725</v>
+      </c>
+      <c r="K42" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="182" t="n">
+        <v>451</v>
+      </c>
+      <c r="M42" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="N42" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O42" s="182" t="n">
+        <v>32898</v>
+      </c>
       <c r="P42" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q42" s="86" t="n"/>
+      <c r="Q42" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 52 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="24" customHeight="1" s="80">
       <c r="A43" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 26/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12040,7 +12040,7 @@
         <v>46290.02230041667</v>
       </c>
       <c r="F42" s="180" t="n">
-        <v>46290.66399692127</v>
+        <v>46290.6639969213</v>
       </c>
       <c r="G42" s="181">
         <f>IF(OR(E42="",F42=""),"",(F42-E42)*24)</f>
@@ -12090,27 +12090,56 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E43" s="180" t="n"/>
-      <c r="F43" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E43" s="180" t="n">
+        <v>46291.02400542824</v>
+      </c>
+      <c r="F43" s="180" t="n">
+        <v>46291.64486558619</v>
+      </c>
       <c r="G43" s="181">
         <f>IF(OR(E43="",F43=""),"",(F43-E43)*24)</f>
         <v/>
       </c>
-      <c r="H43" s="182" t="n"/>
-      <c r="I43" s="182" t="n"/>
-      <c r="J43" s="182" t="n"/>
-      <c r="K43" s="182" t="n"/>
-      <c r="L43" s="182" t="n"/>
-      <c r="M43" s="182" t="n"/>
-      <c r="N43" s="182" t="n"/>
-      <c r="O43" s="182" t="n"/>
+      <c r="H43" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I43" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J43" s="182" t="n">
+        <v>3699</v>
+      </c>
+      <c r="K43" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="182" t="n">
+        <v>417</v>
+      </c>
+      <c r="M43" s="182" t="n">
+        <v>108</v>
+      </c>
+      <c r="N43" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O43" s="182" t="n">
+        <v>32094</v>
+      </c>
       <c r="P43" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q43" s="86" t="n"/>
+      <c r="Q43" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 53 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="24" customHeight="1" s="80">
       <c r="A44" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 27/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12102,7 +12102,7 @@
         <v>46291.02400542824</v>
       </c>
       <c r="F43" s="180" t="n">
-        <v>46291.64486558619</v>
+        <v>46291.64486559028</v>
       </c>
       <c r="G43" s="181">
         <f>IF(OR(E43="",F43=""),"",(F43-E43)*24)</f>
@@ -12152,10 +12152,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E44" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E44" s="180" t="n">
+        <v>46292.02281592875</v>
+      </c>
       <c r="F44" s="180" t="n"/>
       <c r="G44" s="181">
         <f>IF(OR(E44="",F44=""),"",(F44-E44)*24)</f>
@@ -12172,7 +12179,11 @@
       <c r="P44" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q44" s="86" t="n"/>
+      <c r="Q44" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="24" customHeight="1" s="80">
       <c r="A45" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 28/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12152,7 +12152,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -12161,27 +12161,45 @@
         </is>
       </c>
       <c r="E44" s="180" t="n">
-        <v>46292.02281592875</v>
-      </c>
-      <c r="F44" s="180" t="n"/>
+        <v>46292.02281592593</v>
+      </c>
+      <c r="F44" s="180" t="n">
+        <v>46292.64819444445</v>
+      </c>
       <c r="G44" s="181">
         <f>IF(OR(E44="",F44=""),"",(F44-E44)*24)</f>
         <v/>
       </c>
-      <c r="H44" s="182" t="n"/>
-      <c r="I44" s="182" t="n"/>
-      <c r="J44" s="182" t="n"/>
-      <c r="K44" s="182" t="n"/>
-      <c r="L44" s="182" t="n"/>
-      <c r="M44" s="182" t="n"/>
-      <c r="N44" s="182" t="n"/>
-      <c r="O44" s="182" t="n"/>
+      <c r="H44" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I44" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J44" s="182" t="n">
+        <v>3717</v>
+      </c>
+      <c r="K44" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="182" t="n">
+        <v>387</v>
+      </c>
+      <c r="M44" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="N44" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O44" s="182" t="n">
+        <v>34507</v>
+      </c>
       <c r="P44" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q44" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 54 đã đạt terminal state</t>
         </is>
       </c>
     </row>
@@ -12196,27 +12214,56 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E45" s="180" t="n"/>
-      <c r="F45" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E45" s="180" t="n">
+        <v>46293.02343596065</v>
+      </c>
+      <c r="F45" s="180" t="n">
+        <v>46293.66651982639</v>
+      </c>
       <c r="G45" s="181">
         <f>IF(OR(E45="",F45=""),"",(F45-E45)*24)</f>
         <v/>
       </c>
-      <c r="H45" s="182" t="n"/>
-      <c r="I45" s="182" t="n"/>
-      <c r="J45" s="182" t="n"/>
-      <c r="K45" s="182" t="n"/>
-      <c r="L45" s="182" t="n"/>
-      <c r="M45" s="182" t="n"/>
-      <c r="N45" s="182" t="n"/>
-      <c r="O45" s="182" t="n"/>
+      <c r="H45" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I45" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J45" s="182" t="n">
+        <v>3730</v>
+      </c>
+      <c r="K45" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="182" t="n">
+        <v>374</v>
+      </c>
+      <c r="M45" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="N45" s="182" t="n">
+        <v>24</v>
+      </c>
+      <c r="O45" s="182" t="n">
+        <v>34142</v>
+      </c>
       <c r="P45" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q45" s="86" t="n"/>
+      <c r="Q45" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 55 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="24" customHeight="1" s="80">
       <c r="A46" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 29/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12276,27 +12276,56 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E46" s="180" t="n"/>
-      <c r="F46" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E46" s="180" t="n">
+        <v>46294.02265880787</v>
+      </c>
+      <c r="F46" s="180" t="n">
+        <v>46294.65464432501</v>
+      </c>
       <c r="G46" s="181">
         <f>IF(OR(E46="",F46=""),"",(F46-E46)*24)</f>
         <v/>
       </c>
-      <c r="H46" s="182" t="n"/>
-      <c r="I46" s="182" t="n"/>
-      <c r="J46" s="182" t="n"/>
-      <c r="K46" s="182" t="n"/>
-      <c r="L46" s="182" t="n"/>
-      <c r="M46" s="182" t="n"/>
-      <c r="N46" s="182" t="n"/>
-      <c r="O46" s="182" t="n"/>
+      <c r="H46" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I46" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J46" s="182" t="n">
+        <v>3733</v>
+      </c>
+      <c r="K46" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="182" t="n">
+        <v>383</v>
+      </c>
+      <c r="M46" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N46" s="182" t="n">
+        <v>36</v>
+      </c>
+      <c r="O46" s="182" t="n">
+        <v>35263</v>
+      </c>
       <c r="P46" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q46" s="86" t="n"/>
+      <c r="Q46" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 56 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="24" customHeight="1" s="80">
       <c r="A47" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 30/9
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12288,7 +12288,7 @@
         <v>46294.02265880787</v>
       </c>
       <c r="F46" s="180" t="n">
-        <v>46294.65464432501</v>
+        <v>46294.6546443287</v>
       </c>
       <c r="G46" s="181">
         <f>IF(OR(E46="",F46=""),"",(F46-E46)*24)</f>
@@ -12338,27 +12338,56 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E47" s="180" t="n"/>
-      <c r="F47" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E47" s="180" t="n">
+        <v>46295.02316377315</v>
+      </c>
+      <c r="F47" s="180" t="n">
+        <v>46295.67805679525</v>
+      </c>
       <c r="G47" s="181">
         <f>IF(OR(E47="",F47=""),"",(F47-E47)*24)</f>
         <v/>
       </c>
-      <c r="H47" s="182" t="n"/>
-      <c r="I47" s="182" t="n"/>
-      <c r="J47" s="182" t="n"/>
-      <c r="K47" s="182" t="n"/>
-      <c r="L47" s="182" t="n"/>
-      <c r="M47" s="182" t="n"/>
-      <c r="N47" s="182" t="n"/>
-      <c r="O47" s="182" t="n"/>
+      <c r="H47" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I47" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J47" s="182" t="n">
+        <v>3732</v>
+      </c>
+      <c r="K47" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="182" t="n">
+        <v>384</v>
+      </c>
+      <c r="M47" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N47" s="182" t="n">
+        <v>36</v>
+      </c>
+      <c r="O47" s="182" t="n">
+        <v>34518</v>
+      </c>
       <c r="P47" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q47" s="86" t="n"/>
+      <c r="Q47" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 57 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="24" customHeight="1" s="80">
       <c r="A48" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 1/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12350,7 +12350,7 @@
         <v>46295.02316377315</v>
       </c>
       <c r="F47" s="180" t="n">
-        <v>46295.67805679525</v>
+        <v>46295.67805679398</v>
       </c>
       <c r="G47" s="181">
         <f>IF(OR(E47="",F47=""),"",(F47-E47)*24)</f>
@@ -12400,27 +12400,56 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E48" s="180" t="n"/>
-      <c r="F48" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E48" s="180" t="n">
+        <v>46296.0235147338</v>
+      </c>
+      <c r="F48" s="180" t="n">
+        <v>46296.65618110924</v>
+      </c>
       <c r="G48" s="181">
         <f>IF(OR(E48="",F48=""),"",(F48-E48)*24)</f>
         <v/>
       </c>
-      <c r="H48" s="182" t="n"/>
-      <c r="I48" s="182" t="n"/>
-      <c r="J48" s="182" t="n"/>
-      <c r="K48" s="182" t="n"/>
-      <c r="L48" s="182" t="n"/>
-      <c r="M48" s="182" t="n"/>
-      <c r="N48" s="182" t="n"/>
-      <c r="O48" s="182" t="n"/>
+      <c r="H48" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I48" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J48" s="182" t="n">
+        <v>3723</v>
+      </c>
+      <c r="K48" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="182" t="n">
+        <v>369</v>
+      </c>
+      <c r="M48" s="182" t="n">
+        <v>108</v>
+      </c>
+      <c r="N48" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="O48" s="182" t="n">
+        <v>35071</v>
+      </c>
       <c r="P48" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q48" s="86" t="n"/>
+      <c r="Q48" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 58 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="24" customHeight="1" s="80">
       <c r="A49" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 3/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12412,7 +12412,7 @@
         <v>46296.0235147338</v>
       </c>
       <c r="F48" s="180" t="n">
-        <v>46296.65618110924</v>
+        <v>46296.65618111111</v>
       </c>
       <c r="G48" s="181">
         <f>IF(OR(E48="",F48=""),"",(F48-E48)*24)</f>
@@ -12462,27 +12462,56 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E49" s="180" t="n"/>
-      <c r="F49" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E49" s="180" t="n">
+        <v>46297.03225480324</v>
+      </c>
+      <c r="F49" s="180" t="n">
+        <v>46297.67325483797</v>
+      </c>
       <c r="G49" s="181">
         <f>IF(OR(E49="",F49=""),"",(F49-E49)*24)</f>
         <v/>
       </c>
-      <c r="H49" s="182" t="n"/>
-      <c r="I49" s="182" t="n"/>
-      <c r="J49" s="182" t="n"/>
-      <c r="K49" s="182" t="n"/>
-      <c r="L49" s="182" t="n"/>
-      <c r="M49" s="182" t="n"/>
-      <c r="N49" s="182" t="n"/>
-      <c r="O49" s="182" t="n"/>
+      <c r="H49" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I49" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J49" s="182" t="n">
+        <v>3710</v>
+      </c>
+      <c r="K49" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="182" t="n">
+        <v>382</v>
+      </c>
+      <c r="M49" s="182" t="n">
+        <v>108</v>
+      </c>
+      <c r="N49" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="O49" s="182" t="n">
+        <v>34758</v>
+      </c>
       <c r="P49" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q49" s="86" t="n"/>
+      <c r="Q49" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 59 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="24" customHeight="1" s="80">
       <c r="A50" s="177" t="n">
@@ -12495,27 +12524,56 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E50" s="180" t="n"/>
-      <c r="F50" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E50" s="180" t="n">
+        <v>46298.02228471065</v>
+      </c>
+      <c r="F50" s="180" t="n">
+        <v>46298.71745289075</v>
+      </c>
       <c r="G50" s="181">
         <f>IF(OR(E50="",F50=""),"",(F50-E50)*24)</f>
         <v/>
       </c>
-      <c r="H50" s="182" t="n"/>
-      <c r="I50" s="182" t="n"/>
-      <c r="J50" s="182" t="n"/>
-      <c r="K50" s="182" t="n"/>
-      <c r="L50" s="182" t="n"/>
-      <c r="M50" s="182" t="n"/>
-      <c r="N50" s="182" t="n"/>
-      <c r="O50" s="182" t="n"/>
+      <c r="H50" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I50" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J50" s="182" t="n">
+        <v>3702</v>
+      </c>
+      <c r="K50" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="182" t="n">
+        <v>378</v>
+      </c>
+      <c r="M50" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="N50" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="O50" s="182" t="n">
+        <v>33979</v>
+      </c>
       <c r="P50" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q50" s="86" t="n"/>
+      <c r="Q50" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 60 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="24" customHeight="1" s="80">
       <c r="A51" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 4/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12536,7 +12536,7 @@
         <v>46298.02228471065</v>
       </c>
       <c r="F50" s="180" t="n">
-        <v>46298.71745289075</v>
+        <v>46298.71745289352</v>
       </c>
       <c r="G50" s="181">
         <f>IF(OR(E50="",F50=""),"",(F50-E50)*24)</f>
@@ -12586,27 +12586,56 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E51" s="180" t="n"/>
-      <c r="F51" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E51" s="180" t="n">
+        <v>46299.02255300926</v>
+      </c>
+      <c r="F51" s="180" t="n">
+        <v>46299.73926950442</v>
+      </c>
       <c r="G51" s="181">
         <f>IF(OR(E51="",F51=""),"",(F51-E51)*24)</f>
         <v/>
       </c>
-      <c r="H51" s="182" t="n"/>
-      <c r="I51" s="182" t="n"/>
-      <c r="J51" s="182" t="n"/>
-      <c r="K51" s="182" t="n"/>
-      <c r="L51" s="182" t="n"/>
-      <c r="M51" s="182" t="n"/>
-      <c r="N51" s="182" t="n"/>
-      <c r="O51" s="182" t="n"/>
+      <c r="H51" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I51" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J51" s="182" t="n">
+        <v>3682</v>
+      </c>
+      <c r="K51" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="182" t="n">
+        <v>398</v>
+      </c>
+      <c r="M51" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="N51" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="O51" s="182" t="n">
+        <v>33656</v>
+      </c>
       <c r="P51" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q51" s="86" t="n"/>
+      <c r="Q51" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 61 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="24" customHeight="1" s="80">
       <c r="A52" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 5/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12598,7 +12598,7 @@
         <v>46299.02255300926</v>
       </c>
       <c r="F51" s="180" t="n">
-        <v>46299.73926950442</v>
+        <v>46299.73926950232</v>
       </c>
       <c r="G51" s="181">
         <f>IF(OR(E51="",F51=""),"",(F51-E51)*24)</f>
@@ -12648,27 +12648,56 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E52" s="180" t="n"/>
-      <c r="F52" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E52" s="180" t="n">
+        <v>46300.02355754629</v>
+      </c>
+      <c r="F52" s="180" t="n">
+        <v>46300.64516793418</v>
+      </c>
       <c r="G52" s="181">
         <f>IF(OR(E52="",F52=""),"",(F52-E52)*24)</f>
         <v/>
       </c>
-      <c r="H52" s="182" t="n"/>
-      <c r="I52" s="182" t="n"/>
-      <c r="J52" s="182" t="n"/>
-      <c r="K52" s="182" t="n"/>
-      <c r="L52" s="182" t="n"/>
-      <c r="M52" s="182" t="n"/>
-      <c r="N52" s="182" t="n"/>
-      <c r="O52" s="182" t="n"/>
+      <c r="H52" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I52" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J52" s="182" t="n">
+        <v>3696</v>
+      </c>
+      <c r="K52" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="182" t="n">
+        <v>372</v>
+      </c>
+      <c r="M52" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="N52" s="182" t="n">
+        <v>48</v>
+      </c>
+      <c r="O52" s="182" t="n">
+        <v>33856</v>
+      </c>
       <c r="P52" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q52" s="86" t="n"/>
+      <c r="Q52" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 62 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="24" customHeight="1" s="80">
       <c r="A53" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 6/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12660,7 +12660,7 @@
         <v>46300.02355754629</v>
       </c>
       <c r="F52" s="180" t="n">
-        <v>46300.64516793418</v>
+        <v>46300.64516793982</v>
       </c>
       <c r="G52" s="181">
         <f>IF(OR(E52="",F52=""),"",(F52-E52)*24)</f>
@@ -12710,27 +12710,56 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E53" s="180" t="n"/>
-      <c r="F53" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E53" s="180" t="n">
+        <v>46301.02321953703</v>
+      </c>
+      <c r="F53" s="180" t="n">
+        <v>46301.65734304029</v>
+      </c>
       <c r="G53" s="181">
         <f>IF(OR(E53="",F53=""),"",(F53-E53)*24)</f>
         <v/>
       </c>
-      <c r="H53" s="182" t="n"/>
-      <c r="I53" s="182" t="n"/>
-      <c r="J53" s="182" t="n"/>
-      <c r="K53" s="182" t="n"/>
-      <c r="L53" s="182" t="n"/>
-      <c r="M53" s="182" t="n"/>
-      <c r="N53" s="182" t="n"/>
-      <c r="O53" s="182" t="n"/>
+      <c r="H53" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I53" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J53" s="182" t="n">
+        <v>3671</v>
+      </c>
+      <c r="K53" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="182" t="n">
+        <v>397</v>
+      </c>
+      <c r="M53" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="N53" s="182" t="n">
+        <v>60</v>
+      </c>
+      <c r="O53" s="182" t="n">
+        <v>33067</v>
+      </c>
       <c r="P53" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q53" s="86" t="n"/>
+      <c r="Q53" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 63 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="24" customHeight="1" s="80">
       <c r="A54" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 7/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12722,7 +12722,7 @@
         <v>46301.02321953703</v>
       </c>
       <c r="F53" s="180" t="n">
-        <v>46301.65734304029</v>
+        <v>46301.65734304398</v>
       </c>
       <c r="G53" s="181">
         <f>IF(OR(E53="",F53=""),"",(F53-E53)*24)</f>
@@ -12772,27 +12772,56 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E54" s="180" t="n"/>
-      <c r="F54" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E54" s="180" t="n">
+        <v>46302.02248005787</v>
+      </c>
+      <c r="F54" s="180" t="n">
+        <v>46302.64480953976</v>
+      </c>
       <c r="G54" s="181">
         <f>IF(OR(E54="",F54=""),"",(F54-E54)*24)</f>
         <v/>
       </c>
-      <c r="H54" s="182" t="n"/>
-      <c r="I54" s="182" t="n"/>
-      <c r="J54" s="182" t="n"/>
-      <c r="K54" s="182" t="n"/>
-      <c r="L54" s="182" t="n"/>
-      <c r="M54" s="182" t="n"/>
-      <c r="N54" s="182" t="n"/>
-      <c r="O54" s="182" t="n"/>
+      <c r="H54" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I54" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J54" s="182" t="n">
+        <v>3640</v>
+      </c>
+      <c r="K54" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="182" t="n">
+        <v>428</v>
+      </c>
+      <c r="M54" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="N54" s="182" t="n">
+        <v>60</v>
+      </c>
+      <c r="O54" s="182" t="n">
+        <v>33108</v>
+      </c>
       <c r="P54" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q54" s="86" t="n"/>
+      <c r="Q54" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 64 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="24" customHeight="1" s="80">
       <c r="A55" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 11/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -12958,7 +12958,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -12967,27 +12967,45 @@
         </is>
       </c>
       <c r="E57" s="180" t="n">
-        <v>46305.019823493</v>
-      </c>
-      <c r="F57" s="180" t="n"/>
+        <v>46305.01982349537</v>
+      </c>
+      <c r="F57" s="180" t="n">
+        <v>46305.62060153935</v>
+      </c>
       <c r="G57" s="181">
         <f>IF(OR(E57="",F57=""),"",(F57-E57)*24)</f>
         <v/>
       </c>
-      <c r="H57" s="182" t="n"/>
-      <c r="I57" s="182" t="n"/>
-      <c r="J57" s="182" t="n"/>
-      <c r="K57" s="182" t="n"/>
-      <c r="L57" s="182" t="n"/>
-      <c r="M57" s="182" t="n"/>
-      <c r="N57" s="182" t="n"/>
-      <c r="O57" s="182" t="n"/>
+      <c r="H57" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I57" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J57" s="182" t="n">
+        <v>3515</v>
+      </c>
+      <c r="K57" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="182" t="n">
+        <v>505</v>
+      </c>
+      <c r="M57" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N57" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O57" s="182" t="n">
+        <v>31172</v>
+      </c>
       <c r="P57" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q57" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 67 đã đạt terminal state</t>
         </is>
       </c>
     </row>
@@ -13002,27 +13020,56 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E58" s="180" t="n"/>
-      <c r="F58" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E58" s="180" t="n">
+        <v>46306.02451019676</v>
+      </c>
+      <c r="F58" s="180" t="n">
+        <v>46306.63431952207</v>
+      </c>
       <c r="G58" s="181">
         <f>IF(OR(E58="",F58=""),"",(F58-E58)*24)</f>
         <v/>
       </c>
-      <c r="H58" s="182" t="n"/>
-      <c r="I58" s="182" t="n"/>
-      <c r="J58" s="182" t="n"/>
-      <c r="K58" s="182" t="n"/>
-      <c r="L58" s="182" t="n"/>
-      <c r="M58" s="182" t="n"/>
-      <c r="N58" s="182" t="n"/>
-      <c r="O58" s="182" t="n"/>
+      <c r="H58" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I58" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J58" s="182" t="n">
+        <v>3558</v>
+      </c>
+      <c r="K58" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" s="182" t="n">
+        <v>475</v>
+      </c>
+      <c r="M58" s="182" t="n">
+        <v>83</v>
+      </c>
+      <c r="N58" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O58" s="182" t="n">
+        <v>31405</v>
+      </c>
       <c r="P58" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q58" s="86" t="n"/>
+      <c r="Q58" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 68 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="24" customHeight="1" s="80">
       <c r="A59" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 12/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -13032,7 +13032,7 @@
         <v>46306.02451019676</v>
       </c>
       <c r="F58" s="180" t="n">
-        <v>46306.63431952207</v>
+        <v>46306.63431952546</v>
       </c>
       <c r="G58" s="181">
         <f>IF(OR(E58="",F58=""),"",(F58-E58)*24)</f>
@@ -13082,27 +13082,56 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E59" s="180" t="n"/>
-      <c r="F59" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E59" s="180" t="n">
+        <v>46307.02383261574</v>
+      </c>
+      <c r="F59" s="180" t="n">
+        <v>46307.64267200232</v>
+      </c>
       <c r="G59" s="181">
         <f>IF(OR(E59="",F59=""),"",(F59-E59)*24)</f>
         <v/>
       </c>
-      <c r="H59" s="182" t="n"/>
-      <c r="I59" s="182" t="n"/>
-      <c r="J59" s="182" t="n"/>
-      <c r="K59" s="182" t="n"/>
-      <c r="L59" s="182" t="n"/>
-      <c r="M59" s="182" t="n"/>
-      <c r="N59" s="182" t="n"/>
-      <c r="O59" s="182" t="n"/>
+      <c r="H59" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I59" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J59" s="182" t="n">
+        <v>3546</v>
+      </c>
+      <c r="K59" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" s="182" t="n">
+        <v>486</v>
+      </c>
+      <c r="M59" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N59" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O59" s="182" t="n">
+        <v>32980</v>
+      </c>
       <c r="P59" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q59" s="86" t="n"/>
+      <c r="Q59" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 69 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="24" customHeight="1" s="80">
       <c r="A60" s="177" t="n">
@@ -13115,10 +13144,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E60" s="180" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E60" s="180" t="n">
+        <v>46308.01947654462</v>
+      </c>
       <c r="F60" s="180" t="n"/>
       <c r="G60" s="181">
         <f>IF(OR(E60="",F60=""),"",(F60-E60)*24)</f>
@@ -13135,7 +13171,11 @@
       <c r="P60" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q60" s="86" t="n"/>
+      <c r="Q60" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="24" customHeight="1" s="80">
       <c r="A61" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 13/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -13144,7 +13144,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -13153,27 +13153,45 @@
         </is>
       </c>
       <c r="E60" s="180" t="n">
-        <v>46308.01947654462</v>
-      </c>
-      <c r="F60" s="180" t="n"/>
+        <v>46308.01947653935</v>
+      </c>
+      <c r="F60" s="180" t="n">
+        <v>46308.62720308115</v>
+      </c>
       <c r="G60" s="181">
         <f>IF(OR(E60="",F60=""),"",(F60-E60)*24)</f>
         <v/>
       </c>
-      <c r="H60" s="182" t="n"/>
-      <c r="I60" s="182" t="n"/>
-      <c r="J60" s="182" t="n"/>
-      <c r="K60" s="182" t="n"/>
-      <c r="L60" s="182" t="n"/>
-      <c r="M60" s="182" t="n"/>
-      <c r="N60" s="182" t="n"/>
-      <c r="O60" s="182" t="n"/>
+      <c r="H60" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I60" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J60" s="182" t="n">
+        <v>3546</v>
+      </c>
+      <c r="K60" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" s="182" t="n">
+        <v>486</v>
+      </c>
+      <c r="M60" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N60" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O60" s="182" t="n">
+        <v>33235</v>
+      </c>
       <c r="P60" s="182" t="n">
         <v>12</v>
       </c>
       <c r="Q60" s="86" t="inlineStr">
         <is>
-          <t>Scheduled crawl đã tạo durable run; save_artifacts=false</t>
+          <t>Scheduled run 70 đã đạt terminal state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update crawl 19/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -13156,7 +13156,7 @@
         <v>46308.01947653935</v>
       </c>
       <c r="F60" s="180" t="n">
-        <v>46308.62720308115</v>
+        <v>46308.6272030787</v>
       </c>
       <c r="G60" s="181">
         <f>IF(OR(E60="",F60=""),"",(F60-E60)*24)</f>
@@ -13206,27 +13206,56 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E61" s="180" t="n"/>
-      <c r="F61" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="E61" s="180" t="n">
+        <v>46309.02385369213</v>
+      </c>
+      <c r="F61" s="180" t="n">
+        <v>46309.63157362268</v>
+      </c>
       <c r="G61" s="181">
         <f>IF(OR(E61="",F61=""),"",(F61-E61)*24)</f>
         <v/>
       </c>
-      <c r="H61" s="182" t="n"/>
-      <c r="I61" s="182" t="n"/>
-      <c r="J61" s="182" t="n"/>
-      <c r="K61" s="182" t="n"/>
-      <c r="L61" s="182" t="n"/>
-      <c r="M61" s="182" t="n"/>
-      <c r="N61" s="182" t="n"/>
-      <c r="O61" s="182" t="n"/>
+      <c r="H61" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I61" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J61" s="182" t="n">
+        <v>3529</v>
+      </c>
+      <c r="K61" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="182" t="n">
+        <v>503</v>
+      </c>
+      <c r="M61" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N61" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O61" s="182" t="n">
+        <v>32355</v>
+      </c>
       <c r="P61" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q61" s="86" t="n"/>
+      <c r="Q61" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 71 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="24" customHeight="1" s="80">
       <c r="A62" s="177" t="n">
@@ -13239,27 +13268,56 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E62" s="180" t="n"/>
-      <c r="F62" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E62" s="180" t="n">
+        <v>46310.02465560185</v>
+      </c>
+      <c r="F62" s="180" t="n">
+        <v>46310.62056496528</v>
+      </c>
       <c r="G62" s="181">
         <f>IF(OR(E62="",F62=""),"",(F62-E62)*24)</f>
         <v/>
       </c>
-      <c r="H62" s="182" t="n"/>
-      <c r="I62" s="182" t="n"/>
-      <c r="J62" s="182" t="n"/>
-      <c r="K62" s="182" t="n"/>
-      <c r="L62" s="182" t="n"/>
-      <c r="M62" s="182" t="n"/>
-      <c r="N62" s="182" t="n"/>
-      <c r="O62" s="182" t="n"/>
+      <c r="H62" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I62" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J62" s="182" t="n">
+        <v>3501</v>
+      </c>
+      <c r="K62" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" s="182" t="n">
+        <v>531</v>
+      </c>
+      <c r="M62" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N62" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O62" s="182" t="n">
+        <v>31521</v>
+      </c>
       <c r="P62" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q62" s="86" t="n"/>
+      <c r="Q62" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 72 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="24" customHeight="1" s="80">
       <c r="A63" s="177" t="n">
@@ -13272,27 +13330,56 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E63" s="180" t="n"/>
-      <c r="F63" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="E63" s="180" t="n">
+        <v>46311.02530791667</v>
+      </c>
+      <c r="F63" s="180" t="n">
+        <v>46311.63997377315</v>
+      </c>
       <c r="G63" s="181">
         <f>IF(OR(E63="",F63=""),"",(F63-E63)*24)</f>
         <v/>
       </c>
-      <c r="H63" s="182" t="n"/>
-      <c r="I63" s="182" t="n"/>
-      <c r="J63" s="182" t="n"/>
-      <c r="K63" s="182" t="n"/>
-      <c r="L63" s="182" t="n"/>
-      <c r="M63" s="182" t="n"/>
-      <c r="N63" s="182" t="n"/>
-      <c r="O63" s="182" t="n"/>
+      <c r="H63" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I63" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J63" s="182" t="n">
+        <v>3483</v>
+      </c>
+      <c r="K63" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" s="182" t="n">
+        <v>549</v>
+      </c>
+      <c r="M63" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N63" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O63" s="182" t="n">
+        <v>31458</v>
+      </c>
       <c r="P63" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q63" s="86" t="n"/>
+      <c r="Q63" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 73 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="24" customHeight="1" s="80">
       <c r="A64" s="177" t="n">
@@ -13305,27 +13392,56 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E64" s="180" t="n"/>
-      <c r="F64" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="E64" s="180" t="n">
+        <v>46312.01837070602</v>
+      </c>
+      <c r="F64" s="180" t="n">
+        <v>46312.62550892361</v>
+      </c>
       <c r="G64" s="181">
         <f>IF(OR(E64="",F64=""),"",(F64-E64)*24)</f>
         <v/>
       </c>
-      <c r="H64" s="182" t="n"/>
-      <c r="I64" s="182" t="n"/>
-      <c r="J64" s="182" t="n"/>
-      <c r="K64" s="182" t="n"/>
-      <c r="L64" s="182" t="n"/>
-      <c r="M64" s="182" t="n"/>
-      <c r="N64" s="182" t="n"/>
-      <c r="O64" s="182" t="n"/>
+      <c r="H64" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I64" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J64" s="182" t="n">
+        <v>3484</v>
+      </c>
+      <c r="K64" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" s="182" t="n">
+        <v>559</v>
+      </c>
+      <c r="M64" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N64" s="182" t="n">
+        <v>121</v>
+      </c>
+      <c r="O64" s="182" t="n">
+        <v>32164</v>
+      </c>
       <c r="P64" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q64" s="86" t="n"/>
+      <c r="Q64" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 74 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="24" customHeight="1" s="80">
       <c r="A65" s="177" t="n">
@@ -13338,27 +13454,56 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E65" s="180" t="n"/>
-      <c r="F65" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E65" s="180" t="n">
+        <v>46313.0241461574</v>
+      </c>
+      <c r="F65" s="180" t="n">
+        <v>46313.63256355324</v>
+      </c>
       <c r="G65" s="181">
         <f>IF(OR(E65="",F65=""),"",(F65-E65)*24)</f>
         <v/>
       </c>
-      <c r="H65" s="182" t="n"/>
-      <c r="I65" s="182" t="n"/>
-      <c r="J65" s="182" t="n"/>
-      <c r="K65" s="182" t="n"/>
-      <c r="L65" s="182" t="n"/>
-      <c r="M65" s="182" t="n"/>
-      <c r="N65" s="182" t="n"/>
-      <c r="O65" s="182" t="n"/>
+      <c r="H65" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I65" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J65" s="182" t="n">
+        <v>3526</v>
+      </c>
+      <c r="K65" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" s="182" t="n">
+        <v>518</v>
+      </c>
+      <c r="M65" s="182" t="n">
+        <v>84</v>
+      </c>
+      <c r="N65" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="O65" s="182" t="n">
+        <v>32711</v>
+      </c>
       <c r="P65" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q65" s="86" t="n"/>
+      <c r="Q65" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 75 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="24" customHeight="1" s="80">
       <c r="A66" s="177" t="n">
@@ -13371,27 +13516,56 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E66" s="180" t="n"/>
-      <c r="F66" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="E66" s="180" t="n">
+        <v>46314.02472768519</v>
+      </c>
+      <c r="F66" s="180" t="n">
+        <v>46314.6248079803</v>
+      </c>
       <c r="G66" s="181">
         <f>IF(OR(E66="",F66=""),"",(F66-E66)*24)</f>
         <v/>
       </c>
-      <c r="H66" s="182" t="n"/>
-      <c r="I66" s="182" t="n"/>
-      <c r="J66" s="182" t="n"/>
-      <c r="K66" s="182" t="n"/>
-      <c r="L66" s="182" t="n"/>
-      <c r="M66" s="182" t="n"/>
-      <c r="N66" s="182" t="n"/>
-      <c r="O66" s="182" t="n"/>
+      <c r="H66" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I66" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J66" s="182" t="n">
+        <v>3522</v>
+      </c>
+      <c r="K66" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" s="182" t="n">
+        <v>510</v>
+      </c>
+      <c r="M66" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N66" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="O66" s="182" t="n">
+        <v>32007</v>
+      </c>
       <c r="P66" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q66" s="86" t="n"/>
+      <c r="Q66" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 76 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="24" customHeight="1" s="80">
       <c r="A67" s="177" t="n">

</xml_diff>

<commit_message>
feat: update crawl 22/10
</commit_message>
<xml_diff>
--- a/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
+++ b/outputs/crawl-data-planner-20260816/crawl_sampling_master.xlsx
@@ -13528,7 +13528,7 @@
         <v>46314.02472768519</v>
       </c>
       <c r="F66" s="180" t="n">
-        <v>46314.6248079803</v>
+        <v>46314.62480797453</v>
       </c>
       <c r="G66" s="181">
         <f>IF(OR(E66="",F66=""),"",(F66-E66)*24)</f>
@@ -13578,27 +13578,56 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E67" s="180" t="n"/>
-      <c r="F67" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="E67" s="180" t="n">
+        <v>46315.02250773148</v>
+      </c>
+      <c r="F67" s="180" t="n">
+        <v>46315.72886795139</v>
+      </c>
       <c r="G67" s="181">
         <f>IF(OR(E67="",F67=""),"",(F67-E67)*24)</f>
         <v/>
       </c>
-      <c r="H67" s="182" t="n"/>
-      <c r="I67" s="182" t="n"/>
-      <c r="J67" s="182" t="n"/>
-      <c r="K67" s="182" t="n"/>
-      <c r="L67" s="182" t="n"/>
-      <c r="M67" s="182" t="n"/>
-      <c r="N67" s="182" t="n"/>
-      <c r="O67" s="182" t="n"/>
+      <c r="H67" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I67" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J67" s="182" t="n">
+        <v>3500</v>
+      </c>
+      <c r="K67" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" s="182" t="n">
+        <v>520</v>
+      </c>
+      <c r="M67" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N67" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O67" s="182" t="n">
+        <v>31514</v>
+      </c>
       <c r="P67" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q67" s="86" t="n"/>
+      <c r="Q67" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 77 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="24" customHeight="1" s="80">
       <c r="A68" s="177" t="n">
@@ -13611,27 +13640,56 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E68" s="180" t="n"/>
-      <c r="F68" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="E68" s="180" t="n">
+        <v>46316.02113340278</v>
+      </c>
+      <c r="F68" s="180" t="n">
+        <v>46316.64976929398</v>
+      </c>
       <c r="G68" s="181">
         <f>IF(OR(E68="",F68=""),"",(F68-E68)*24)</f>
         <v/>
       </c>
-      <c r="H68" s="182" t="n"/>
-      <c r="I68" s="182" t="n"/>
-      <c r="J68" s="182" t="n"/>
-      <c r="K68" s="182" t="n"/>
-      <c r="L68" s="182" t="n"/>
-      <c r="M68" s="182" t="n"/>
-      <c r="N68" s="182" t="n"/>
-      <c r="O68" s="182" t="n"/>
+      <c r="H68" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I68" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J68" s="182" t="n">
+        <v>3490</v>
+      </c>
+      <c r="K68" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="182" t="n">
+        <v>530</v>
+      </c>
+      <c r="M68" s="182" t="n">
+        <v>96</v>
+      </c>
+      <c r="N68" s="182" t="n">
+        <v>132</v>
+      </c>
+      <c r="O68" s="182" t="n">
+        <v>32175</v>
+      </c>
       <c r="P68" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q68" s="86" t="n"/>
+      <c r="Q68" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 78 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="24" customHeight="1" s="80">
       <c r="A69" s="177" t="n">
@@ -13644,27 +13702,56 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="E69" s="180" t="n"/>
-      <c r="F69" s="180" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="E69" s="180" t="n">
+        <v>46317.02122927083</v>
+      </c>
+      <c r="F69" s="180" t="n">
+        <v>46317.59491939712</v>
+      </c>
       <c r="G69" s="181">
         <f>IF(OR(E69="",F69=""),"",(F69-E69)*24)</f>
         <v/>
       </c>
-      <c r="H69" s="182" t="n"/>
-      <c r="I69" s="182" t="n"/>
-      <c r="J69" s="182" t="n"/>
-      <c r="K69" s="182" t="n"/>
-      <c r="L69" s="182" t="n"/>
-      <c r="M69" s="182" t="n"/>
-      <c r="N69" s="182" t="n"/>
-      <c r="O69" s="182" t="n"/>
+      <c r="H69" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="I69" s="182" t="n">
+        <v>4248</v>
+      </c>
+      <c r="J69" s="182" t="n">
+        <v>3299</v>
+      </c>
+      <c r="K69" s="182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="182" t="n">
+        <v>517</v>
+      </c>
+      <c r="M69" s="182" t="n">
+        <v>312</v>
+      </c>
+      <c r="N69" s="182" t="n">
+        <v>120</v>
+      </c>
+      <c r="O69" s="182" t="n">
+        <v>30417</v>
+      </c>
       <c r="P69" s="182" t="n">
         <v>12</v>
       </c>
-      <c r="Q69" s="86" t="n"/>
+      <c r="Q69" s="86" t="inlineStr">
+        <is>
+          <t>Scheduled run 79 đã đạt terminal state</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="24" customHeight="1" s="80">
       <c r="A70" s="177" t="n">

</xml_diff>